<commit_message>
change the UOM column sequence
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -160,7 +160,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -199,25 +202,25 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:S16" totalsRowShown="0">
   <autoFilter ref="A1:S16"/>
   <tableColumns count="19">
-    <tableColumn id="1" name="No" dataDxfId="7"/>
+    <tableColumn id="1" name="No" dataDxfId="8"/>
     <tableColumn id="15" name="Item code"/>
     <tableColumn id="16" name="Item Description"/>
     <tableColumn id="21" name="Type"/>
     <tableColumn id="20" name="Brand"/>
     <tableColumn id="19" name="Measurement"/>
     <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="price" dataDxfId="6"/>
-    <tableColumn id="3" name="start date" dataDxfId="5"/>
-    <tableColumn id="4" name="end date" dataDxfId="4"/>
+    <tableColumn id="2" name="price" dataDxfId="7"/>
+    <tableColumn id="3" name="start date" dataDxfId="6"/>
+    <tableColumn id="4" name="end date" dataDxfId="5"/>
+    <tableColumn id="7" name="UOM" dataDxfId="0"/>
     <tableColumn id="5" name="additional item description"/>
-    <tableColumn id="6" name="Frequency" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM"/>
+    <tableColumn id="6" name="Frequency" dataDxfId="4"/>
     <tableColumn id="8" name="Model Number"/>
     <tableColumn id="9" name="SKU Number"/>
     <tableColumn id="10" name="Manufacturer's Part Number"/>
-    <tableColumn id="11" name="Min order" dataDxfId="2"/>
-    <tableColumn id="12" name="Max Order" dataDxfId="1"/>
-    <tableColumn id="13" name="Lead Time" dataDxfId="0"/>
+    <tableColumn id="11" name="Min order" dataDxfId="3"/>
+    <tableColumn id="12" name="Max Order" dataDxfId="2"/>
+    <tableColumn id="13" name="Lead Time" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -585,7 +588,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="6" customWidth="1"/>
@@ -597,18 +600,18 @@
     <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="11.5703125" style="5" customWidth="1"/>
     <col min="10" max="10" width="11" style="5" customWidth="1"/>
-    <col min="11" max="11" width="27.140625" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" style="4" customWidth="1"/>
-    <col min="13" max="13" width="7.85546875" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" customWidth="1"/>
-    <col min="15" max="15" width="14.42578125" customWidth="1"/>
-    <col min="16" max="16" width="28.42578125" customWidth="1"/>
-    <col min="17" max="17" width="12" style="4" customWidth="1"/>
-    <col min="18" max="18" width="12.5703125" style="4" customWidth="1"/>
-    <col min="19" max="19" width="12.140625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="27.140625" customWidth="1"/>
+    <col min="13" max="13" width="12.42578125" style="4" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" customWidth="1"/>
+    <col min="16" max="16" width="14.42578125" customWidth="1"/>
+    <col min="17" max="17" width="28.42578125" customWidth="1"/>
+    <col min="18" max="18" width="12" style="4" customWidth="1"/>
+    <col min="19" max="19" width="12.5703125" style="4" customWidth="1"/>
+    <col min="20" max="20" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>16</v>
       </c>
@@ -640,13 +643,13 @@
         <v>2</v>
       </c>
       <c r="K1" t="s">
+        <v>4</v>
+      </c>
+      <c r="L1" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="M1" t="s">
-        <v>4</v>
       </c>
       <c r="N1" t="s">
         <v>5</v>
@@ -666,55 +669,88 @@
       <c r="S1" s="4" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M3" s="1"/>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M4" s="1"/>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M5" s="1"/>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M6" s="1"/>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M7" s="1"/>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M8" s="1"/>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M9" s="1"/>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M10" s="1"/>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M11" s="1"/>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M12" s="1"/>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M13" s="1"/>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M14" s="1"/>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M15" s="1"/>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="M16" s="1"/>
+      <c r="T1"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="Q2" s="4"/>
+      <c r="T2"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K3" s="1"/>
+      <c r="Q3" s="4"/>
+      <c r="T3"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K4" s="1"/>
+      <c r="Q4" s="4"/>
+      <c r="T4"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K5" s="1"/>
+      <c r="Q5" s="4"/>
+      <c r="T5"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K6" s="1"/>
+      <c r="Q6" s="4"/>
+      <c r="T6"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K7" s="1"/>
+      <c r="Q7" s="4"/>
+      <c r="T7"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K8" s="1"/>
+      <c r="Q8" s="4"/>
+      <c r="T8"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K9" s="1"/>
+      <c r="Q9" s="4"/>
+      <c r="T9"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K10" s="1"/>
+      <c r="Q10" s="4"/>
+      <c r="T10"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K11" s="1"/>
+      <c r="Q11" s="4"/>
+      <c r="T11"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K12" s="1"/>
+      <c r="Q12" s="4"/>
+      <c r="T12"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K13" s="1"/>
+      <c r="Q13" s="4"/>
+      <c r="T13"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K14" s="1"/>
+      <c r="Q14" s="4"/>
+      <c r="T14"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K15" s="1"/>
+      <c r="Q15" s="4"/>
+      <c r="T15"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="K16" s="1"/>
+      <c r="Q16" s="4"/>
+      <c r="T16"/>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="L1:L1048576 Q1:S1048576">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="M1:M1048576 Q1:S16 R17:T1048576">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1:J1048576">
@@ -734,7 +770,7 @@
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>M1:M1048576</xm:sqref>
+          <xm:sqref>K1:K1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
*** empty log message ***
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -128,12 +128,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -148,7 +154,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -156,13 +162,16 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="9">
     <dxf>
-      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -174,7 +183,7 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
@@ -212,15 +221,15 @@
     <tableColumn id="2" name="price" dataDxfId="7"/>
     <tableColumn id="3" name="start date" dataDxfId="6"/>
     <tableColumn id="4" name="end date" dataDxfId="5"/>
-    <tableColumn id="7" name="UOM" dataDxfId="0"/>
+    <tableColumn id="7" name="UOM" dataDxfId="4"/>
     <tableColumn id="5" name="additional item description"/>
-    <tableColumn id="6" name="Frequency" dataDxfId="4"/>
+    <tableColumn id="6" name="Frequency" dataDxfId="3"/>
     <tableColumn id="8" name="Model Number"/>
     <tableColumn id="9" name="SKU Number"/>
     <tableColumn id="10" name="Manufacturer's Part Number"/>
-    <tableColumn id="11" name="Min order" dataDxfId="3"/>
-    <tableColumn id="12" name="Max Order" dataDxfId="2"/>
-    <tableColumn id="13" name="Lead Time" dataDxfId="1"/>
+    <tableColumn id="11" name="Min order" dataDxfId="2"/>
+    <tableColumn id="12" name="Max Order" dataDxfId="1"/>
+    <tableColumn id="13" name="Lead Time" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -633,16 +642,16 @@
       <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="9" t="s">
         <v>4</v>
       </c>
       <c r="L1" t="s">

</xml_diff>

<commit_message>
SIR #3664, renamed "Lead Time" to "Delivery Term"
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -58,9 +58,6 @@
     <t>Max Order</t>
   </si>
   <si>
-    <t>Lead Time</t>
-  </si>
-  <si>
     <t>Frequency</t>
   </si>
   <si>
@@ -104,6 +101,9 @@
   </si>
   <si>
     <t>Item Description</t>
+  </si>
+  <si>
+    <t>Delivery Term</t>
   </si>
 </sst>
 </file>
@@ -229,7 +229,7 @@
     <tableColumn id="10" name="Manufacturer's Part Number"/>
     <tableColumn id="11" name="Min order" dataDxfId="2"/>
     <tableColumn id="12" name="Max Order" dataDxfId="1"/>
-    <tableColumn id="13" name="Lead Time" dataDxfId="0"/>
+    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -530,7 +530,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2"/>
     </row>
@@ -539,7 +539,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -547,7 +547,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -555,7 +555,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -563,7 +563,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -571,7 +571,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -579,7 +579,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -587,7 +587,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -614,33 +614,33 @@
     <col min="13" max="13" width="12.42578125" style="4" customWidth="1"/>
     <col min="15" max="15" width="16.7109375" customWidth="1"/>
     <col min="16" max="16" width="14.42578125" customWidth="1"/>
-    <col min="17" max="17" width="28.42578125" customWidth="1"/>
-    <col min="18" max="18" width="12" style="4" customWidth="1"/>
-    <col min="19" max="19" width="12.5703125" style="4" customWidth="1"/>
+    <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>25</v>
-      </c>
       <c r="D1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>0</v>
@@ -658,7 +658,7 @@
         <v>3</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N1" t="s">
         <v>5</v>
@@ -676,7 +676,7 @@
         <v>9</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="T1"/>
     </row>
@@ -755,17 +755,18 @@
       <c r="T16"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="M1:M1048576 Q1:S16 R17:T1048576">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="M1:M1048576 R17:T1048576 Q1:R16 S2:S16">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1:J1048576">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="S1"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
Bug fix for Bug #3664
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="240" windowWidth="8595" windowHeight="5265" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="2472" windowWidth="17928" windowHeight="4536" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -21,12 +21,13 @@
     <definedName name="ZonalDistrictList">INDEX(#REF!,0,MATCH(#REF!,StateList,0))</definedName>
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="124519"/>
+  <oleSize ref="A1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t>price</t>
   </si>
@@ -37,9 +38,6 @@
     <t>end date</t>
   </si>
   <si>
-    <t>additional item description</t>
-  </si>
-  <si>
     <t>UOM</t>
   </si>
   <si>
@@ -49,18 +47,9 @@
     <t>SKU Number</t>
   </si>
   <si>
-    <t>Manufacturer's Part Number</t>
-  </si>
-  <si>
     <t>Min order</t>
   </si>
   <si>
-    <t>Max Order</t>
-  </si>
-  <si>
-    <t>Frequency</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
@@ -100,20 +89,26 @@
     <t>Item code</t>
   </si>
   <si>
-    <t>Item Description</t>
-  </si>
-  <si>
     <t>Delivery Term</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item </t>
+  </si>
+  <si>
+    <t>Manufacturing Part No.</t>
+  </si>
+  <si>
+    <t>Additional Description</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -169,13 +164,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
+  <dxfs count="7">
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -208,27 +197,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:S16" totalsRowShown="0">
-  <autoFilter ref="A1:S16"/>
-  <tableColumns count="19">
-    <tableColumn id="1" name="No" dataDxfId="8"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16"/>
+  <tableColumns count="17">
+    <tableColumn id="1" name="No" dataDxfId="6"/>
     <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item Description"/>
+    <tableColumn id="16" name="Item "/>
     <tableColumn id="21" name="Type"/>
     <tableColumn id="20" name="Brand"/>
     <tableColumn id="19" name="Measurement"/>
     <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="price" dataDxfId="7"/>
-    <tableColumn id="3" name="start date" dataDxfId="6"/>
-    <tableColumn id="4" name="end date" dataDxfId="5"/>
-    <tableColumn id="7" name="UOM" dataDxfId="4"/>
-    <tableColumn id="5" name="additional item description"/>
-    <tableColumn id="6" name="Frequency" dataDxfId="3"/>
+    <tableColumn id="2" name="price" dataDxfId="5"/>
+    <tableColumn id="3" name="start date" dataDxfId="4"/>
+    <tableColumn id="4" name="end date" dataDxfId="3"/>
+    <tableColumn id="7" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" name="Additional Description"/>
     <tableColumn id="8" name="Model Number"/>
     <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturer's Part Number"/>
-    <tableColumn id="11" name="Min order" dataDxfId="2"/>
-    <tableColumn id="12" name="Max Order" dataDxfId="1"/>
+    <tableColumn id="10" name="Manufacturing Part No."/>
+    <tableColumn id="11" name="Min order" dataDxfId="1"/>
     <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -310,7 +297,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -345,7 +331,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -521,73 +506,73 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="5.5703125" customWidth="1"/>
+    <col min="1" max="1" width="5.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" s="3">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6" s="3">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7" s="3">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
       <c r="A8" s="3">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -596,51 +581,50 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:R16"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="16.5703125" style="6" customWidth="1"/>
-    <col min="2" max="3" width="16.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" style="5" customWidth="1"/>
+    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" style="5" customWidth="1"/>
     <col min="10" max="10" width="11" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.85546875" customWidth="1"/>
-    <col min="12" max="12" width="27.140625" customWidth="1"/>
-    <col min="13" max="13" width="12.42578125" style="4" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" customWidth="1"/>
-    <col min="16" max="16" width="14.42578125" customWidth="1"/>
-    <col min="17" max="17" width="12.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12.140625" style="4" customWidth="1"/>
+    <col min="11" max="11" width="7.88671875" customWidth="1"/>
+    <col min="12" max="12" width="23.109375" customWidth="1"/>
+    <col min="13" max="14" width="16.6640625" customWidth="1"/>
+    <col min="15" max="15" width="22.88671875" customWidth="1"/>
+    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18">
       <c r="A1" s="6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>0</v>
@@ -652,121 +636,115 @@
         <v>2</v>
       </c>
       <c r="K1" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="M1" t="s">
         <v>4</v>
-      </c>
-      <c r="L1" t="s">
-        <v>3</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>10</v>
       </c>
       <c r="N1" t="s">
         <v>5</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="P1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="P1" t="s">
-        <v>7</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="T1"/>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="Q2" s="4"/>
-      <c r="T2"/>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="R1"/>
+    </row>
+    <row r="2" spans="1:18">
+      <c r="P2" s="4"/>
+      <c r="R2"/>
+    </row>
+    <row r="3" spans="1:18">
       <c r="K3" s="1"/>
-      <c r="Q3" s="4"/>
-      <c r="T3"/>
-    </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P3" s="4"/>
+      <c r="R3"/>
+    </row>
+    <row r="4" spans="1:18">
       <c r="K4" s="1"/>
-      <c r="Q4" s="4"/>
-      <c r="T4"/>
-    </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P4" s="4"/>
+      <c r="R4"/>
+    </row>
+    <row r="5" spans="1:18">
       <c r="K5" s="1"/>
-      <c r="Q5" s="4"/>
-      <c r="T5"/>
-    </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P5" s="4"/>
+      <c r="R5"/>
+    </row>
+    <row r="6" spans="1:18">
       <c r="K6" s="1"/>
-      <c r="Q6" s="4"/>
-      <c r="T6"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P6" s="4"/>
+      <c r="R6"/>
+    </row>
+    <row r="7" spans="1:18">
       <c r="K7" s="1"/>
-      <c r="Q7" s="4"/>
-      <c r="T7"/>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P7" s="4"/>
+      <c r="R7"/>
+    </row>
+    <row r="8" spans="1:18">
       <c r="K8" s="1"/>
-      <c r="Q8" s="4"/>
-      <c r="T8"/>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P8" s="4"/>
+      <c r="R8"/>
+    </row>
+    <row r="9" spans="1:18">
       <c r="K9" s="1"/>
-      <c r="Q9" s="4"/>
-      <c r="T9"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P9" s="4"/>
+      <c r="R9"/>
+    </row>
+    <row r="10" spans="1:18">
       <c r="K10" s="1"/>
-      <c r="Q10" s="4"/>
-      <c r="T10"/>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P10" s="4"/>
+      <c r="R10"/>
+    </row>
+    <row r="11" spans="1:18">
       <c r="K11" s="1"/>
-      <c r="Q11" s="4"/>
-      <c r="T11"/>
-    </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P11" s="4"/>
+      <c r="R11"/>
+    </row>
+    <row r="12" spans="1:18">
       <c r="K12" s="1"/>
-      <c r="Q12" s="4"/>
-      <c r="T12"/>
-    </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P12" s="4"/>
+      <c r="R12"/>
+    </row>
+    <row r="13" spans="1:18">
       <c r="K13" s="1"/>
-      <c r="Q13" s="4"/>
-      <c r="T13"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P13" s="4"/>
+      <c r="R13"/>
+    </row>
+    <row r="14" spans="1:18">
       <c r="K14" s="1"/>
-      <c r="Q14" s="4"/>
-      <c r="T14"/>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P14" s="4"/>
+      <c r="R14"/>
+    </row>
+    <row r="15" spans="1:18">
       <c r="K15" s="1"/>
-      <c r="Q15" s="4"/>
-      <c r="T15"/>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="P15" s="4"/>
+      <c r="R15"/>
+    </row>
+    <row r="16" spans="1:18">
       <c r="K16" s="1"/>
-      <c r="Q16" s="4"/>
-      <c r="T16"/>
+      <c r="P16" s="4"/>
+      <c r="R16"/>
     </row>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="M1:M1048576 R17:T1048576 Q1:R16 S2:S16">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1:J1048576">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="S1"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -789,1005 +767,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="1" max="1" width="9.109375" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:2">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:2">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:2">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:2">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:2">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:2">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:2">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:2">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:2">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:2">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:2">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:2">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:2">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:2">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:2">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:2">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:2">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:2">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:2">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:2">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:2">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:2">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:2">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:2">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:2">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:2">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:2">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:2">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:2">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:2">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:2">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:2">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:2">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:2">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:2">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:2">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:2">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:2">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:2">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:2">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:2">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:2">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:2">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:2">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:2">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:2">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:2">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:2">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:2">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:2">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:2">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:2">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:2">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:2">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:2">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:2">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:2">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:2">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:2">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:2">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:2">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="2:2">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="2:2">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="2:2">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="2:2">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="2:2">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="2:2">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="2:2">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="2:2">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="2:2">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="2:2">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="2:2">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="2:2">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="2:2">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="2:2">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="2:2">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="2:2">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:2">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:2">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:2">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:2">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="2:2">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:2">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:2">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:2">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:2">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:2">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:2">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:2">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:2">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:2">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:2">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:2">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="2:2">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="2:2">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="2:2">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="2:2">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="2:2">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="2:2">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="2:2">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="2:2">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="2:2">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="2:2">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="2:2">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="2:2">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="2:2">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="2:2">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="2:2">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="2:2">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="2:2">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="2:2">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="2:2">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="2:2">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="2:2">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="2:2">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="2:2">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="2:2">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="2:2">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="2:2">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="2:2">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="2:2">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="2:2">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="2:2">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="2:2">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="2:2">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="2:2">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="2:2">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="2:2">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="2:2">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="2:2">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="2:2">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="2:2">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="2:2">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="2:2">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="2:2">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="2:2">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="2:2">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="2:2">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="2:2">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="2:2">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="2:2">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="2:2">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="2:2">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="2:2">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="2:2">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="2:2">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="2:2">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="151" spans="2:2">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="152" spans="2:2">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="153" spans="2:2">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="154" spans="2:2">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="155" spans="2:2">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="156" spans="2:2">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="157" spans="2:2">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="158" spans="2:2">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="159" spans="2:2">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="160" spans="2:2">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="161" spans="2:2">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="162" spans="2:2">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="2:2">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="2:2">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="165" spans="2:2">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="166" spans="2:2">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="167" spans="2:2">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="168" spans="2:2">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="169" spans="2:2">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="170" spans="2:2">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="171" spans="2:2">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="172" spans="2:2">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="173" spans="2:2">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="174" spans="2:2">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="175" spans="2:2">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="176" spans="2:2">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="177" spans="2:2">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="178" spans="2:2">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="179" spans="2:2">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="180" spans="2:2">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="181" spans="2:2">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="182" spans="2:2">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="183" spans="2:2">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="184" spans="2:2">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="185" spans="2:2">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="186" spans="2:2">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="187" spans="2:2">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="188" spans="2:2">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="189" spans="2:2">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="190" spans="2:2">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="191" spans="2:2">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="192" spans="2:2">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="193" spans="2:2">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="194" spans="2:2">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="195" spans="2:2">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="196" spans="2:2">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="197" spans="2:2">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="198" spans="2:2">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="199" spans="2:2">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="200" spans="2:2">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="201" spans="2:2">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="202" spans="2:2">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="203" spans="2:2">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="204" spans="2:2">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="205" spans="2:2">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="206" spans="2:2">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="207" spans="2:2">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="208" spans="2:2">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="209" spans="2:2">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="210" spans="2:2">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="211" spans="2:2">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="212" spans="2:2">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="213" spans="2:2">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="214" spans="2:2">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="215" spans="2:2">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="216" spans="2:2">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="217" spans="2:2">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="218" spans="2:2">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="219" spans="2:2">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="220" spans="2:2">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="221" spans="2:2">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="222" spans="2:2">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="223" spans="2:2">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="224" spans="2:2">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="225" spans="2:2">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="226" spans="2:2">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="227" spans="2:2">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="228" spans="2:2">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="229" spans="2:2">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="230" spans="2:2">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="231" spans="2:2">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="232" spans="2:2">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="233" spans="2:2">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="234" spans="2:2">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="235" spans="2:2">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="236" spans="2:2">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="237" spans="2:2">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="238" spans="2:2">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="239" spans="2:2">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="240" spans="2:2">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="241" spans="2:2">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="242" spans="2:2">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="243" spans="2:2">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="244" spans="2:2">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="245" spans="2:2">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="246" spans="2:2">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="247" spans="2:2">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="248" spans="2:2">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="249" spans="2:2">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="250" spans="2:2">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="251" spans="2:2">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="252" spans="2:2">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="253" spans="2:2">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="254" spans="2:2">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="255" spans="2:2">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="256" spans="2:2">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="257" spans="2:2">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="258" spans="2:2">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="259" spans="2:2">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="260" spans="2:2">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="261" spans="2:2">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="262" spans="2:2">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="263" spans="2:2">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="264" spans="2:2">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="265" spans="2:2">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="266" spans="2:2">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="267" spans="2:2">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="268" spans="2:2">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="269" spans="2:2">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="270" spans="2:2">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="271" spans="2:2">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="272" spans="2:2">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="273" spans="2:2">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="274" spans="2:2">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="275" spans="2:2">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="276" spans="2:2">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="277" spans="2:2">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="278" spans="2:2">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="279" spans="2:2">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="280" spans="2:2">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="281" spans="2:2">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="282" spans="2:2">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="283" spans="2:2">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="284" spans="2:2">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="285" spans="2:2">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="286" spans="2:2">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="287" spans="2:2">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="288" spans="2:2">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="289" spans="2:2">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="290" spans="2:2">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="291" spans="2:2">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="292" spans="2:2">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="293" spans="2:2">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="294" spans="2:2">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="295" spans="2:2">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="296" spans="2:2">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="297" spans="2:2">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="298" spans="2:2">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="299" spans="2:2">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="300" spans="2:2">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="301" spans="2:2">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="302" spans="2:2">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="303" spans="2:2">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="304" spans="2:2">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="305" spans="2:2">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="306" spans="2:2">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="307" spans="2:2">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="308" spans="2:2">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="309" spans="2:2">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="310" spans="2:2">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="311" spans="2:2">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="312" spans="2:2">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="313" spans="2:2">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="314" spans="2:2">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="315" spans="2:2">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="316" spans="2:2">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="317" spans="2:2">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="318" spans="2:2">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="319" spans="2:2">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="320" spans="2:2">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="321" spans="2:2">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="322" spans="2:2">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="323" spans="2:2">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="324" spans="2:2">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="325" spans="2:2">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="326" spans="2:2">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="327" spans="2:2">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="328" spans="2:2">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="329" spans="2:2">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="330" spans="2:2">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="331" spans="2:2">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modified column names for Bug#3664
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2472" windowWidth="17928" windowHeight="4536" activeTab="1"/>
+    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -29,15 +29,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
-    <t>price</t>
-  </si>
-  <si>
-    <t>start date</t>
-  </si>
-  <si>
-    <t>end date</t>
-  </si>
-  <si>
     <t>UOM</t>
   </si>
   <si>
@@ -99,6 +90,15 @@
   </si>
   <si>
     <t>Additional Description</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Start Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>End Date(dd/MM/yyyy)</t>
   </si>
 </sst>
 </file>
@@ -207,9 +207,9 @@
     <tableColumn id="20" name="Brand"/>
     <tableColumn id="19" name="Measurement"/>
     <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="price" dataDxfId="5"/>
-    <tableColumn id="3" name="start date" dataDxfId="4"/>
-    <tableColumn id="4" name="end date" dataDxfId="3"/>
+    <tableColumn id="2" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
     <tableColumn id="7" name="UOM" dataDxfId="2"/>
     <tableColumn id="5" name="Additional Description"/>
     <tableColumn id="8" name="Model Number"/>
@@ -515,7 +515,7 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
@@ -524,7 +524,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -532,7 +532,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -540,7 +540,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -548,7 +548,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -556,7 +556,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:2">
@@ -564,7 +564,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:2">
@@ -572,7 +572,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -593,8 +593,8 @@
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
-    <col min="9" max="9" width="11.5546875" style="5" customWidth="1"/>
-    <col min="10" max="10" width="11" style="5" customWidth="1"/>
+    <col min="9" max="9" width="26" style="5" customWidth="1"/>
+    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
     <col min="11" max="11" width="7.88671875" customWidth="1"/>
     <col min="12" max="12" width="23.109375" customWidth="1"/>
     <col min="13" max="14" width="16.6640625" customWidth="1"/>
@@ -606,55 +606,55 @@
   <sheetData>
     <row r="1" spans="1:18">
       <c r="A1" s="6" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" t="s">
+        <v>2</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="K1" s="9" t="s">
+      <c r="P1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" t="s">
-        <v>4</v>
-      </c>
-      <c r="N1" t="s">
-        <v>5</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="Q1" s="4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="R1"/>
     </row>
@@ -733,18 +733,22 @@
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576">
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
+      <formula1>0</formula1>
+    </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>

</xml_diff>

<commit_message>
Enhancement #30457 : Section B � CMCD part A-E
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17670" windowHeight="5370" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -22,7 +27,6 @@
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -104,11 +108,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,7 +168,29 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -187,10 +213,18 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -200,23 +234,23 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
   <autoFilter ref="A1:Q16"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="6"/>
+    <tableColumn id="1" name="No" dataDxfId="8"/>
     <tableColumn id="15" name="Item code"/>
     <tableColumn id="16" name="Item "/>
     <tableColumn id="21" name="Type"/>
     <tableColumn id="20" name="Brand"/>
     <tableColumn id="19" name="Measurement"/>
     <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="5"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM" dataDxfId="2"/>
+    <tableColumn id="2" name="Price" dataDxfId="7"/>
+    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="6"/>
+    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="5"/>
+    <tableColumn id="7" name="UOM" dataDxfId="4"/>
     <tableColumn id="5" name="Additional Description"/>
     <tableColumn id="8" name="Model Number"/>
     <tableColumn id="9" name="SKU Number"/>
     <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="1"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
+    <tableColumn id="11" name="Min order" dataDxfId="3"/>
+    <tableColumn id="13" name="Delivery Term" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -265,7 +299,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,9 +331,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -331,6 +366,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -506,20 +542,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -527,7 +563,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -535,7 +571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -543,7 +579,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -551,7 +587,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -559,7 +595,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -567,7 +603,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -581,30 +617,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" customWidth="1"/>
-    <col min="13" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="22.88671875" customWidth="1"/>
-    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
+    <col min="13" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
@@ -638,7 +674,7 @@
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="9" t="s">
         <v>20</v>
       </c>
       <c r="M1" t="s">
@@ -658,76 +694,76 @@
       </c>
       <c r="R1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P2" s="4"/>
       <c r="R2"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="P3" s="4"/>
       <c r="R3"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K4" s="1"/>
       <c r="P4" s="4"/>
       <c r="R4"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K5" s="1"/>
       <c r="P5" s="4"/>
       <c r="R5"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K6" s="1"/>
       <c r="P6" s="4"/>
       <c r="R6"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K7" s="1"/>
       <c r="P7" s="4"/>
       <c r="R7"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K8" s="1"/>
       <c r="P8" s="4"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K9" s="1"/>
       <c r="P9" s="4"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K10" s="1"/>
       <c r="P10" s="4"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K11" s="1"/>
       <c r="P11" s="4"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K12" s="1"/>
       <c r="P12" s="4"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K13" s="1"/>
       <c r="P13" s="4"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K14" s="1"/>
       <c r="P14" s="4"/>
       <c r="R14"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
       <c r="P15" s="4"/>
       <c r="R15"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
       <c r="P16" s="4"/>
       <c r="R16"/>
@@ -771,1005 +807,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
merge HEAD->release SIT : #30457
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="17670" windowHeight="5370" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -22,7 +27,6 @@
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -104,11 +108,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,7 +168,29 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -187,10 +213,18 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+      <tableStyleElement type="wholeTable" dxfId="1"/>
+      <tableStyleElement type="headerRow" dxfId="0"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -200,23 +234,23 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
   <autoFilter ref="A1:Q16"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="6"/>
+    <tableColumn id="1" name="No" dataDxfId="8"/>
     <tableColumn id="15" name="Item code"/>
     <tableColumn id="16" name="Item "/>
     <tableColumn id="21" name="Type"/>
     <tableColumn id="20" name="Brand"/>
     <tableColumn id="19" name="Measurement"/>
     <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="5"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM" dataDxfId="2"/>
+    <tableColumn id="2" name="Price" dataDxfId="7"/>
+    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="6"/>
+    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="5"/>
+    <tableColumn id="7" name="UOM" dataDxfId="4"/>
     <tableColumn id="5" name="Additional Description"/>
     <tableColumn id="8" name="Model Number"/>
     <tableColumn id="9" name="SKU Number"/>
     <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="1"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
+    <tableColumn id="11" name="Min order" dataDxfId="3"/>
+    <tableColumn id="13" name="Delivery Term" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -265,7 +299,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,9 +331,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -331,6 +366,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -506,20 +542,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -527,7 +563,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -535,7 +571,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -543,7 +579,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -551,7 +587,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -559,7 +595,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -567,7 +603,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -581,30 +617,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" customWidth="1"/>
-    <col min="13" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="22.88671875" customWidth="1"/>
-    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
+    <col min="13" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
@@ -638,7 +674,7 @@
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="9" t="s">
         <v>20</v>
       </c>
       <c r="M1" t="s">
@@ -658,76 +694,76 @@
       </c>
       <c r="R1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P2" s="4"/>
       <c r="R2"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="P3" s="4"/>
       <c r="R3"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K4" s="1"/>
       <c r="P4" s="4"/>
       <c r="R4"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K5" s="1"/>
       <c r="P5" s="4"/>
       <c r="R5"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K6" s="1"/>
       <c r="P6" s="4"/>
       <c r="R6"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K7" s="1"/>
       <c r="P7" s="4"/>
       <c r="R7"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K8" s="1"/>
       <c r="P8" s="4"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K9" s="1"/>
       <c r="P9" s="4"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K10" s="1"/>
       <c r="P10" s="4"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K11" s="1"/>
       <c r="P11" s="4"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K12" s="1"/>
       <c r="P12" s="4"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K13" s="1"/>
       <c r="P13" s="4"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K14" s="1"/>
       <c r="P14" s="4"/>
       <c r="R14"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
       <c r="P15" s="4"/>
       <c r="R15"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
       <c r="P16" s="4"/>
       <c r="R16"/>
@@ -771,1005 +807,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#30457 - change wording
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382896F1-0A0F-4533-808A-30DC33985247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17670" windowHeight="5370" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -93,9 +94,6 @@
     <t>Manufacturing Part No.</t>
   </si>
   <si>
-    <t>Additional Description</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
@@ -103,12 +101,15 @@
   </si>
   <si>
     <t>End Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Basic Specification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
@@ -170,6 +171,27 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -191,32 +213,11 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="0"/>
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -231,26 +232,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
-  <autoFilter ref="A1:Q16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="8"/>
-    <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item "/>
-    <tableColumn id="21" name="Type"/>
-    <tableColumn id="20" name="Brand"/>
-    <tableColumn id="19" name="Measurement"/>
-    <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="7"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="6"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="5"/>
-    <tableColumn id="7" name="UOM" dataDxfId="4"/>
-    <tableColumn id="5" name="Additional Description"/>
-    <tableColumn id="8" name="Model Number"/>
-    <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="3"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Item code"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Item "/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Type"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Brand"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Measurement"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colour"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Basic Specification"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Model Number"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SKU Number"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Manufacturing Part No."/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Min order" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -332,6 +333,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -367,6 +385,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -542,7 +577,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -617,7 +652,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -663,19 +698,19 @@
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>1</v>
@@ -769,22 +804,19 @@
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
+  <dataValidations count="5">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1" xr:uid="{00000000-0002-0000-0100-000005000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -794,7 +826,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
@@ -807,7 +839,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B331"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
merge HEAD->release SIT : #30457 merged by muin
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382896F1-0A0F-4533-808A-30DC33985247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17670" windowHeight="5370" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -93,9 +94,6 @@
     <t>Manufacturing Part No.</t>
   </si>
   <si>
-    <t>Additional Description</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
@@ -103,12 +101,15 @@
   </si>
   <si>
     <t>End Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Basic Specification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
@@ -170,6 +171,27 @@
   </cellStyles>
   <dxfs count="9">
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -191,32 +213,11 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
-      <tableStyleElement type="wholeTable" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="0"/>
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -231,26 +232,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
-  <autoFilter ref="A1:Q16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="8"/>
-    <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item "/>
-    <tableColumn id="21" name="Type"/>
-    <tableColumn id="20" name="Brand"/>
-    <tableColumn id="19" name="Measurement"/>
-    <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="7"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="6"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="5"/>
-    <tableColumn id="7" name="UOM" dataDxfId="4"/>
-    <tableColumn id="5" name="Additional Description"/>
-    <tableColumn id="8" name="Model Number"/>
-    <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="3"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Item code"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Item "/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Type"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Brand"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Measurement"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colour"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Basic Specification"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Model Number"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SKU Number"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Manufacturing Part No."/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Min order" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -332,6 +333,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -367,6 +385,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -542,7 +577,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -617,7 +652,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -663,19 +698,19 @@
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
       <c r="L1" s="9" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>1</v>
@@ -769,22 +804,19 @@
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
+  <dataValidations count="5">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1" xr:uid="{00000000-0002-0000-0100-000005000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -794,7 +826,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
@@ -807,7 +839,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B331"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
merge release-sit -> release-prd-uat : #30457
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382896F1-0A0F-4533-808A-30DC33985247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -22,7 +28,6 @@
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -89,9 +94,6 @@
     <t>Manufacturing Part No.</t>
   </si>
   <si>
-    <t>Additional Description</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
@@ -99,16 +101,19 @@
   </si>
   <si>
     <t>End Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Basic Specification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,7 +169,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -186,37 +191,67 @@
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
-  <autoFilter ref="A1:Q16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="6"/>
-    <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item "/>
-    <tableColumn id="21" name="Type"/>
-    <tableColumn id="20" name="Brand"/>
-    <tableColumn id="19" name="Measurement"/>
-    <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="5"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM" dataDxfId="2"/>
-    <tableColumn id="5" name="Additional Description"/>
-    <tableColumn id="8" name="Model Number"/>
-    <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="1"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Item code"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Item "/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Type"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Brand"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Measurement"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colour"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Basic Specification"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Model Number"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SKU Number"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Manufacturing Part No."/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Min order" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -265,7 +300,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,9 +332,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -331,6 +384,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -506,20 +577,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -527,7 +598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -535,7 +606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -543,7 +614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -551,7 +622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -559,7 +630,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -567,7 +638,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -581,30 +652,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" customWidth="1"/>
-    <col min="13" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="22.88671875" customWidth="1"/>
-    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
+    <col min="13" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
@@ -627,19 +698,19 @@
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
+      <c r="L1" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>1</v>
@@ -658,97 +729,94 @@
       </c>
       <c r="R1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P2" s="4"/>
       <c r="R2"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="P3" s="4"/>
       <c r="R3"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K4" s="1"/>
       <c r="P4" s="4"/>
       <c r="R4"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K5" s="1"/>
       <c r="P5" s="4"/>
       <c r="R5"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K6" s="1"/>
       <c r="P6" s="4"/>
       <c r="R6"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K7" s="1"/>
       <c r="P7" s="4"/>
       <c r="R7"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K8" s="1"/>
       <c r="P8" s="4"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K9" s="1"/>
       <c r="P9" s="4"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K10" s="1"/>
       <c r="P10" s="4"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K11" s="1"/>
       <c r="P11" s="4"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K12" s="1"/>
       <c r="P12" s="4"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K13" s="1"/>
       <c r="P13" s="4"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K14" s="1"/>
       <c r="P14" s="4"/>
       <c r="R14"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
       <c r="P15" s="4"/>
       <c r="R15"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
       <c r="P16" s="4"/>
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
+  <dataValidations count="5">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1" xr:uid="{00000000-0002-0000-0100-000005000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -758,7 +826,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
@@ -771,1005 +839,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
merge release-prd-uat > release-pre-prd : #30457
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382896F1-0A0F-4533-808A-30DC33985247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -22,7 +28,6 @@
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -89,9 +94,6 @@
     <t>Manufacturing Part No.</t>
   </si>
   <si>
-    <t>Additional Description</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
@@ -99,16 +101,19 @@
   </si>
   <si>
     <t>End Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Basic Specification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,7 +169,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -186,37 +191,67 @@
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
-  <autoFilter ref="A1:Q16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="6"/>
-    <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item "/>
-    <tableColumn id="21" name="Type"/>
-    <tableColumn id="20" name="Brand"/>
-    <tableColumn id="19" name="Measurement"/>
-    <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="5"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM" dataDxfId="2"/>
-    <tableColumn id="5" name="Additional Description"/>
-    <tableColumn id="8" name="Model Number"/>
-    <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="1"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Item code"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Item "/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Type"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Brand"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Measurement"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colour"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Basic Specification"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Model Number"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SKU Number"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Manufacturing Part No."/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Min order" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -265,7 +300,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,9 +332,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -331,6 +384,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -506,20 +577,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -527,7 +598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -535,7 +606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -543,7 +614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -551,7 +622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -559,7 +630,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -567,7 +638,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -581,30 +652,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" customWidth="1"/>
-    <col min="13" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="22.88671875" customWidth="1"/>
-    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
+    <col min="13" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
@@ -627,19 +698,19 @@
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
+      <c r="L1" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>1</v>
@@ -658,97 +729,94 @@
       </c>
       <c r="R1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P2" s="4"/>
       <c r="R2"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="P3" s="4"/>
       <c r="R3"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K4" s="1"/>
       <c r="P4" s="4"/>
       <c r="R4"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K5" s="1"/>
       <c r="P5" s="4"/>
       <c r="R5"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K6" s="1"/>
       <c r="P6" s="4"/>
       <c r="R6"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K7" s="1"/>
       <c r="P7" s="4"/>
       <c r="R7"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K8" s="1"/>
       <c r="P8" s="4"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K9" s="1"/>
       <c r="P9" s="4"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K10" s="1"/>
       <c r="P10" s="4"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K11" s="1"/>
       <c r="P11" s="4"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K12" s="1"/>
       <c r="P12" s="4"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K13" s="1"/>
       <c r="P13" s="4"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K14" s="1"/>
       <c r="P14" s="4"/>
       <c r="R14"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
       <c r="P15" s="4"/>
       <c r="R15"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
       <c r="P16" s="4"/>
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
+  <dataValidations count="5">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1" xr:uid="{00000000-0002-0000-0100-000005000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -758,7 +826,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
@@ -771,1005 +839,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FEAT CMCD PRE-PRD #30457
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382896F1-0A0F-4533-808A-30DC33985247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -22,7 +28,6 @@
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -89,9 +94,6 @@
     <t>Manufacturing Part No.</t>
   </si>
   <si>
-    <t>Additional Description</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
@@ -99,16 +101,19 @@
   </si>
   <si>
     <t>End Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Basic Specification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,7 +169,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -186,37 +191,67 @@
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
-  <autoFilter ref="A1:Q16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="6"/>
-    <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item "/>
-    <tableColumn id="21" name="Type"/>
-    <tableColumn id="20" name="Brand"/>
-    <tableColumn id="19" name="Measurement"/>
-    <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="5"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM" dataDxfId="2"/>
-    <tableColumn id="5" name="Additional Description"/>
-    <tableColumn id="8" name="Model Number"/>
-    <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="1"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Item code"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Item "/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Type"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Brand"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Measurement"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colour"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Basic Specification"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Model Number"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SKU Number"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Manufacturing Part No."/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Min order" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -265,7 +300,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,9 +332,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -331,6 +384,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -506,20 +577,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -527,7 +598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -535,7 +606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -543,7 +614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -551,7 +622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -559,7 +630,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -567,7 +638,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -581,30 +652,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" customWidth="1"/>
-    <col min="13" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="22.88671875" customWidth="1"/>
-    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
+    <col min="13" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
@@ -627,19 +698,19 @@
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
+      <c r="L1" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>1</v>
@@ -658,97 +729,94 @@
       </c>
       <c r="R1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P2" s="4"/>
       <c r="R2"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="P3" s="4"/>
       <c r="R3"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K4" s="1"/>
       <c r="P4" s="4"/>
       <c r="R4"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K5" s="1"/>
       <c r="P5" s="4"/>
       <c r="R5"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K6" s="1"/>
       <c r="P6" s="4"/>
       <c r="R6"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K7" s="1"/>
       <c r="P7" s="4"/>
       <c r="R7"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K8" s="1"/>
       <c r="P8" s="4"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K9" s="1"/>
       <c r="P9" s="4"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K10" s="1"/>
       <c r="P10" s="4"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K11" s="1"/>
       <c r="P11" s="4"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K12" s="1"/>
       <c r="P12" s="4"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K13" s="1"/>
       <c r="P13" s="4"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K14" s="1"/>
       <c r="P14" s="4"/>
       <c r="R14"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
       <c r="P15" s="4"/>
       <c r="R15"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
       <c r="P16" s="4"/>
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
+  <dataValidations count="5">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1" xr:uid="{00000000-0002-0000-0100-000005000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -758,7 +826,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
@@ -771,1005 +839,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
merge release-pre-prd-> release-prd : #30457
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382896F1-0A0F-4533-808A-30DC33985247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -22,7 +28,6 @@
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -89,9 +94,6 @@
     <t>Manufacturing Part No.</t>
   </si>
   <si>
-    <t>Additional Description</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
@@ -99,16 +101,19 @@
   </si>
   <si>
     <t>End Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Basic Specification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,7 +169,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -186,37 +191,67 @@
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
-  <autoFilter ref="A1:Q16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="6"/>
-    <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item "/>
-    <tableColumn id="21" name="Type"/>
-    <tableColumn id="20" name="Brand"/>
-    <tableColumn id="19" name="Measurement"/>
-    <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="5"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM" dataDxfId="2"/>
-    <tableColumn id="5" name="Additional Description"/>
-    <tableColumn id="8" name="Model Number"/>
-    <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="1"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Item code"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Item "/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Type"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Brand"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Measurement"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colour"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Basic Specification"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Model Number"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SKU Number"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Manufacturing Part No."/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Min order" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -265,7 +300,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,9 +332,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -331,6 +384,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -506,20 +577,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -527,7 +598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -535,7 +606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -543,7 +614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -551,7 +622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -559,7 +630,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -567,7 +638,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -581,30 +652,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" customWidth="1"/>
-    <col min="13" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="22.88671875" customWidth="1"/>
-    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
+    <col min="13" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
@@ -627,19 +698,19 @@
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
+      <c r="L1" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>1</v>
@@ -658,97 +729,94 @@
       </c>
       <c r="R1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P2" s="4"/>
       <c r="R2"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="P3" s="4"/>
       <c r="R3"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K4" s="1"/>
       <c r="P4" s="4"/>
       <c r="R4"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K5" s="1"/>
       <c r="P5" s="4"/>
       <c r="R5"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K6" s="1"/>
       <c r="P6" s="4"/>
       <c r="R6"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K7" s="1"/>
       <c r="P7" s="4"/>
       <c r="R7"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K8" s="1"/>
       <c r="P8" s="4"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K9" s="1"/>
       <c r="P9" s="4"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K10" s="1"/>
       <c r="P10" s="4"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K11" s="1"/>
       <c r="P11" s="4"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K12" s="1"/>
       <c r="P12" s="4"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K13" s="1"/>
       <c r="P13" s="4"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K14" s="1"/>
       <c r="P14" s="4"/>
       <c r="R14"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
       <c r="P15" s="4"/>
       <c r="R15"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
       <c r="P16" s="4"/>
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
+  <dataValidations count="5">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1" xr:uid="{00000000-0002-0000-0100-000005000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -758,7 +826,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
@@ -771,1005 +839,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FEAT CMCD PRD #30457
</commit_message>
<xml_diff>
--- a/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
+++ b/portlets/NGeP-portlet/docroot/excelUpload/Catalogue-offline-template.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\installation_material\working_folder\NGeP4\liferay-plugins-sdk-6.1.1\portlets\NGeP-portlet\docroot\excelUpload\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{382896F1-0A0F-4533-808A-30DC33985247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="veryHidden" xWindow="0" yWindow="0" windowWidth="17664" windowHeight="5364" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assumption" sheetId="5" r:id="rId1"/>
@@ -22,7 +28,6 @@
     <definedName name="zonalPricingType">Sheet!#REF!</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
-  <oleSize ref="A1"/>
 </workbook>
 </file>
 
@@ -89,9 +94,6 @@
     <t>Manufacturing Part No.</t>
   </si>
   <si>
-    <t>Additional Description</t>
-  </si>
-  <si>
     <t>Price</t>
   </si>
   <si>
@@ -99,16 +101,19 @@
   </si>
   <si>
     <t>End Date(dd/MM/yyyy)</t>
+  </si>
+  <si>
+    <t>Basic Specification</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14409]dd/mm/yy;@"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -164,7 +169,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="9">
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
@@ -186,37 +191,67 @@
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFD7D7D7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
+      <tableStyleElement type="wholeTable" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+    </tableStyle>
+  </tableStyles>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
-  <autoFilter ref="A1:Q16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:Q16" totalsRowShown="0">
+  <autoFilter ref="A1:Q16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="No" dataDxfId="6"/>
-    <tableColumn id="15" name="Item code"/>
-    <tableColumn id="16" name="Item "/>
-    <tableColumn id="21" name="Type"/>
-    <tableColumn id="20" name="Brand"/>
-    <tableColumn id="19" name="Measurement"/>
-    <tableColumn id="18" name="Colour"/>
-    <tableColumn id="2" name="Price" dataDxfId="5"/>
-    <tableColumn id="3" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
-    <tableColumn id="4" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
-    <tableColumn id="7" name="UOM" dataDxfId="2"/>
-    <tableColumn id="5" name="Additional Description"/>
-    <tableColumn id="8" name="Model Number"/>
-    <tableColumn id="9" name="SKU Number"/>
-    <tableColumn id="10" name="Manufacturing Part No."/>
-    <tableColumn id="11" name="Min order" dataDxfId="1"/>
-    <tableColumn id="13" name="Delivery Term" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="No" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Item code"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="Item "/>
+    <tableColumn id="21" xr3:uid="{00000000-0010-0000-0000-000015000000}" name="Type"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Brand"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Measurement"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Colour"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Price" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Start Date(dd/MM/yyyy)" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="End Date(dd/MM/yyyy)" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="UOM" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Basic Specification"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Model Number"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="SKU Number"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Manufacturing Part No."/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Min order" dataDxfId="1"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Delivery Term" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -265,7 +300,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -297,9 +332,27 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -331,6 +384,24 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -506,20 +577,20 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="2"/>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -527,7 +598,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -535,7 +606,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -543,7 +614,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -551,7 +622,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -559,7 +630,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -567,7 +638,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -581,30 +652,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9.44140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="6" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="9.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.42578125" style="4" customWidth="1"/>
     <col min="9" max="9" width="26" style="5" customWidth="1"/>
-    <col min="10" max="10" width="21.77734375" style="5" customWidth="1"/>
-    <col min="11" max="11" width="7.88671875" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" customWidth="1"/>
-    <col min="13" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="22.88671875" customWidth="1"/>
-    <col min="16" max="16" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="15.88671875" style="4" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.109375" style="4" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" style="5" customWidth="1"/>
+    <col min="11" max="11" width="7.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" customWidth="1"/>
+    <col min="13" max="14" width="16.7109375" customWidth="1"/>
+    <col min="15" max="15" width="22.85546875" customWidth="1"/>
+    <col min="16" max="16" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="15.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.140625" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
@@ -627,19 +698,19 @@
         <v>7</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>22</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>23</v>
       </c>
       <c r="K1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>20</v>
+      <c r="L1" s="9" t="s">
+        <v>23</v>
       </c>
       <c r="M1" t="s">
         <v>1</v>
@@ -658,97 +729,94 @@
       </c>
       <c r="R1"/>
     </row>
-    <row r="2" spans="1:18">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="P2" s="4"/>
       <c r="R2"/>
     </row>
-    <row r="3" spans="1:18">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K3" s="1"/>
       <c r="P3" s="4"/>
       <c r="R3"/>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K4" s="1"/>
       <c r="P4" s="4"/>
       <c r="R4"/>
     </row>
-    <row r="5" spans="1:18">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K5" s="1"/>
       <c r="P5" s="4"/>
       <c r="R5"/>
     </row>
-    <row r="6" spans="1:18">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K6" s="1"/>
       <c r="P6" s="4"/>
       <c r="R6"/>
     </row>
-    <row r="7" spans="1:18">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K7" s="1"/>
       <c r="P7" s="4"/>
       <c r="R7"/>
     </row>
-    <row r="8" spans="1:18">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K8" s="1"/>
       <c r="P8" s="4"/>
       <c r="R8"/>
     </row>
-    <row r="9" spans="1:18">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K9" s="1"/>
       <c r="P9" s="4"/>
       <c r="R9"/>
     </row>
-    <row r="10" spans="1:18">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K10" s="1"/>
       <c r="P10" s="4"/>
       <c r="R10"/>
     </row>
-    <row r="11" spans="1:18">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K11" s="1"/>
       <c r="P11" s="4"/>
       <c r="R11"/>
     </row>
-    <row r="12" spans="1:18">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K12" s="1"/>
       <c r="P12" s="4"/>
       <c r="R12"/>
     </row>
-    <row r="13" spans="1:18">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K13" s="1"/>
       <c r="P13" s="4"/>
       <c r="R13"/>
     </row>
-    <row r="14" spans="1:18">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K14" s="1"/>
       <c r="P14" s="4"/>
       <c r="R14"/>
     </row>
-    <row r="15" spans="1:18">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K15" s="1"/>
       <c r="P15" s="4"/>
       <c r="R15"/>
     </row>
-    <row r="16" spans="1:18">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="K16" s="1"/>
       <c r="P16" s="4"/>
       <c r="R16"/>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576">
+  <dataValidations count="5">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q2:Q16 P1:P16 Q17:R1048576" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1"/>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H2:H1048576">
+    <dataValidation operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="Q1" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
+    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1:H1048576" xr:uid="{00000000-0002-0000-0100-000002000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576">
+    <dataValidation type="date" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I2:I1048576 J2:J1048576" xr:uid="{00000000-0002-0000-0100-000003000000}">
       <formula1>1</formula1>
       <formula2>402133</formula2>
     </dataValidation>
-    <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Only numeric values allowed. Please enter valid input." sqref="H1">
-      <formula1>0</formula1>
-    </dataValidation>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Invalid date." sqref="I1 J1" xr:uid="{00000000-0002-0000-0100-000005000000}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="4294967293" r:id="rId1"/>
@@ -758,7 +826,7 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0100-000006000000}">
           <x14:formula1>
             <xm:f>Sheet!$A:$A</xm:f>
           </x14:formula1>
@@ -771,1005 +839,1005 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B331"/>
-  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.109375" style="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
     <col min="2" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="2:2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" s="1"/>
     </row>
-    <row r="3" spans="2:2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="2:2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="2:2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B5" s="1"/>
     </row>
-    <row r="6" spans="2:2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B6" s="1"/>
     </row>
-    <row r="7" spans="2:2">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B7" s="1"/>
     </row>
-    <row r="8" spans="2:2">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B8" s="1"/>
     </row>
-    <row r="9" spans="2:2">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B9" s="1"/>
     </row>
-    <row r="10" spans="2:2">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B10" s="1"/>
     </row>
-    <row r="11" spans="2:2">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B11" s="1"/>
     </row>
-    <row r="12" spans="2:2">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B12" s="1"/>
     </row>
-    <row r="13" spans="2:2">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B13" s="1"/>
     </row>
-    <row r="14" spans="2:2">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B14" s="1"/>
     </row>
-    <row r="15" spans="2:2">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" s="1"/>
     </row>
-    <row r="16" spans="2:2">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B16" s="1"/>
     </row>
-    <row r="17" spans="2:2">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="1"/>
     </row>
-    <row r="18" spans="2:2">
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="1"/>
     </row>
-    <row r="19" spans="2:2">
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B19" s="1"/>
     </row>
-    <row r="20" spans="2:2">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B20" s="1"/>
     </row>
-    <row r="21" spans="2:2">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B21" s="1"/>
     </row>
-    <row r="22" spans="2:2">
+    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B22" s="1"/>
     </row>
-    <row r="23" spans="2:2">
+    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B23" s="1"/>
     </row>
-    <row r="24" spans="2:2">
+    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B24" s="1"/>
     </row>
-    <row r="25" spans="2:2">
+    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B25" s="1"/>
     </row>
-    <row r="26" spans="2:2">
+    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B26" s="1"/>
     </row>
-    <row r="27" spans="2:2">
+    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B27" s="1"/>
     </row>
-    <row r="28" spans="2:2">
+    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B28" s="1"/>
     </row>
-    <row r="29" spans="2:2">
+    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B29" s="1"/>
     </row>
-    <row r="30" spans="2:2">
+    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B30" s="1"/>
     </row>
-    <row r="31" spans="2:2">
+    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B31" s="1"/>
     </row>
-    <row r="32" spans="2:2">
+    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B32" s="1"/>
     </row>
-    <row r="33" spans="2:2">
+    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B33" s="1"/>
     </row>
-    <row r="34" spans="2:2">
+    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B34" s="1"/>
     </row>
-    <row r="35" spans="2:2">
+    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B35" s="1"/>
     </row>
-    <row r="36" spans="2:2">
+    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B36" s="1"/>
     </row>
-    <row r="37" spans="2:2">
+    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B37" s="1"/>
     </row>
-    <row r="38" spans="2:2">
+    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B38" s="1"/>
     </row>
-    <row r="39" spans="2:2">
+    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B39" s="1"/>
     </row>
-    <row r="40" spans="2:2">
+    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B40" s="1"/>
     </row>
-    <row r="41" spans="2:2">
+    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B41" s="1"/>
     </row>
-    <row r="42" spans="2:2">
+    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
     </row>
-    <row r="43" spans="2:2">
+    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B43" s="1"/>
     </row>
-    <row r="44" spans="2:2">
+    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B44" s="1"/>
     </row>
-    <row r="45" spans="2:2">
+    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B45" s="1"/>
     </row>
-    <row r="46" spans="2:2">
+    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B46" s="1"/>
     </row>
-    <row r="47" spans="2:2">
+    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B47" s="1"/>
     </row>
-    <row r="48" spans="2:2">
+    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B48" s="1"/>
     </row>
-    <row r="49" spans="2:2">
+    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B49" s="1"/>
     </row>
-    <row r="50" spans="2:2">
+    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B50" s="1"/>
     </row>
-    <row r="51" spans="2:2">
+    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B51" s="1"/>
     </row>
-    <row r="52" spans="2:2">
+    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B52" s="1"/>
     </row>
-    <row r="53" spans="2:2">
+    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B53" s="1"/>
     </row>
-    <row r="54" spans="2:2">
+    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B54" s="1"/>
     </row>
-    <row r="55" spans="2:2">
+    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B55" s="1"/>
     </row>
-    <row r="56" spans="2:2">
+    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B56" s="1"/>
     </row>
-    <row r="57" spans="2:2">
+    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B57" s="1"/>
     </row>
-    <row r="58" spans="2:2">
+    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B58" s="1"/>
     </row>
-    <row r="59" spans="2:2">
+    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B59" s="1"/>
     </row>
-    <row r="60" spans="2:2">
+    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B60" s="1"/>
     </row>
-    <row r="61" spans="2:2">
+    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B61" s="1"/>
     </row>
-    <row r="62" spans="2:2">
+    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B62" s="1"/>
     </row>
-    <row r="63" spans="2:2">
+    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B63" s="1"/>
     </row>
-    <row r="64" spans="2:2">
+    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B64" s="1"/>
     </row>
-    <row r="65" spans="2:2">
+    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B65" s="1"/>
     </row>
-    <row r="66" spans="2:2">
+    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B66" s="1"/>
     </row>
-    <row r="67" spans="2:2">
+    <row r="67" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B67" s="1"/>
     </row>
-    <row r="68" spans="2:2">
+    <row r="68" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B68" s="1"/>
     </row>
-    <row r="69" spans="2:2">
+    <row r="69" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B69" s="1"/>
     </row>
-    <row r="70" spans="2:2">
+    <row r="70" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B70" s="1"/>
     </row>
-    <row r="71" spans="2:2">
+    <row r="71" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B71" s="1"/>
     </row>
-    <row r="72" spans="2:2">
+    <row r="72" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B72" s="1"/>
     </row>
-    <row r="73" spans="2:2">
+    <row r="73" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B73" s="1"/>
     </row>
-    <row r="74" spans="2:2">
+    <row r="74" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B74" s="1"/>
     </row>
-    <row r="75" spans="2:2">
+    <row r="75" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B75" s="1"/>
     </row>
-    <row r="76" spans="2:2">
+    <row r="76" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B76" s="1"/>
     </row>
-    <row r="77" spans="2:2">
+    <row r="77" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B77" s="1"/>
     </row>
-    <row r="78" spans="2:2">
+    <row r="78" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B78" s="1"/>
     </row>
-    <row r="79" spans="2:2">
+    <row r="79" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B79" s="1"/>
     </row>
-    <row r="80" spans="2:2">
+    <row r="80" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B80" s="1"/>
     </row>
-    <row r="81" spans="2:2">
+    <row r="81" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B81" s="1"/>
     </row>
-    <row r="82" spans="2:2">
+    <row r="82" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B82" s="1"/>
     </row>
-    <row r="83" spans="2:2">
+    <row r="83" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B83" s="1"/>
     </row>
-    <row r="84" spans="2:2">
+    <row r="84" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B84" s="1"/>
     </row>
-    <row r="85" spans="2:2">
+    <row r="85" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B85" s="1"/>
     </row>
-    <row r="86" spans="2:2">
+    <row r="86" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B86" s="1"/>
     </row>
-    <row r="87" spans="2:2">
+    <row r="87" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B87" s="1"/>
     </row>
-    <row r="88" spans="2:2">
+    <row r="88" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B88" s="1"/>
     </row>
-    <row r="89" spans="2:2">
+    <row r="89" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B89" s="1"/>
     </row>
-    <row r="90" spans="2:2">
+    <row r="90" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B90" s="1"/>
     </row>
-    <row r="91" spans="2:2">
+    <row r="91" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B91" s="1"/>
     </row>
-    <row r="92" spans="2:2">
+    <row r="92" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B92" s="1"/>
     </row>
-    <row r="93" spans="2:2">
+    <row r="93" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B93" s="1"/>
     </row>
-    <row r="94" spans="2:2">
+    <row r="94" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B94" s="1"/>
     </row>
-    <row r="95" spans="2:2">
+    <row r="95" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B95" s="1"/>
     </row>
-    <row r="96" spans="2:2">
+    <row r="96" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B96" s="1"/>
     </row>
-    <row r="97" spans="2:2">
+    <row r="97" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B97" s="1"/>
     </row>
-    <row r="98" spans="2:2">
+    <row r="98" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B98" s="1"/>
     </row>
-    <row r="99" spans="2:2">
+    <row r="99" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B99" s="1"/>
     </row>
-    <row r="100" spans="2:2">
+    <row r="100" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B100" s="1"/>
     </row>
-    <row r="101" spans="2:2">
+    <row r="101" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B101" s="1"/>
     </row>
-    <row r="102" spans="2:2">
+    <row r="102" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B102" s="1"/>
     </row>
-    <row r="103" spans="2:2">
+    <row r="103" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B103" s="1"/>
     </row>
-    <row r="104" spans="2:2">
+    <row r="104" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B104" s="1"/>
     </row>
-    <row r="105" spans="2:2">
+    <row r="105" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B105" s="1"/>
     </row>
-    <row r="106" spans="2:2">
+    <row r="106" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B106" s="1"/>
     </row>
-    <row r="107" spans="2:2">
+    <row r="107" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B107" s="1"/>
     </row>
-    <row r="108" spans="2:2">
+    <row r="108" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B108" s="1"/>
     </row>
-    <row r="109" spans="2:2">
+    <row r="109" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B109" s="1"/>
     </row>
-    <row r="110" spans="2:2">
+    <row r="110" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B110" s="1"/>
     </row>
-    <row r="111" spans="2:2">
+    <row r="111" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B111" s="1"/>
     </row>
-    <row r="112" spans="2:2">
+    <row r="112" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B112" s="1"/>
     </row>
-    <row r="113" spans="2:2">
+    <row r="113" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B113" s="1"/>
     </row>
-    <row r="114" spans="2:2">
+    <row r="114" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B114" s="1"/>
     </row>
-    <row r="115" spans="2:2">
+    <row r="115" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B115" s="1"/>
     </row>
-    <row r="116" spans="2:2">
+    <row r="116" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B116" s="1"/>
     </row>
-    <row r="117" spans="2:2">
+    <row r="117" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B117" s="1"/>
     </row>
-    <row r="118" spans="2:2">
+    <row r="118" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B118" s="1"/>
     </row>
-    <row r="119" spans="2:2">
+    <row r="119" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B119" s="1"/>
     </row>
-    <row r="120" spans="2:2">
+    <row r="120" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B120" s="1"/>
     </row>
-    <row r="121" spans="2:2">
+    <row r="121" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B121" s="1"/>
     </row>
-    <row r="122" spans="2:2">
+    <row r="122" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B122" s="1"/>
     </row>
-    <row r="123" spans="2:2">
+    <row r="123" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B123" s="1"/>
     </row>
-    <row r="124" spans="2:2">
+    <row r="124" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B124" s="1"/>
     </row>
-    <row r="125" spans="2:2">
+    <row r="125" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B125" s="1"/>
     </row>
-    <row r="126" spans="2:2">
+    <row r="126" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B126" s="1"/>
     </row>
-    <row r="127" spans="2:2">
+    <row r="127" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B127" s="1"/>
     </row>
-    <row r="128" spans="2:2">
+    <row r="128" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B128" s="1"/>
     </row>
-    <row r="129" spans="2:2">
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B129" s="1"/>
     </row>
-    <row r="130" spans="2:2">
+    <row r="130" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B130" s="1"/>
     </row>
-    <row r="131" spans="2:2">
+    <row r="131" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B131" s="1"/>
     </row>
-    <row r="132" spans="2:2">
+    <row r="132" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B132" s="1"/>
     </row>
-    <row r="133" spans="2:2">
+    <row r="133" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B133" s="1"/>
     </row>
-    <row r="134" spans="2:2">
+    <row r="134" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B134" s="1"/>
     </row>
-    <row r="135" spans="2:2">
+    <row r="135" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B135" s="1"/>
     </row>
-    <row r="136" spans="2:2">
+    <row r="136" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B136" s="1"/>
     </row>
-    <row r="137" spans="2:2">
+    <row r="137" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B137" s="1"/>
     </row>
-    <row r="138" spans="2:2">
+    <row r="138" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B138" s="1"/>
     </row>
-    <row r="139" spans="2:2">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
-    <row r="140" spans="2:2">
+    <row r="140" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B140" s="1"/>
     </row>
-    <row r="141" spans="2:2">
+    <row r="141" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B141" s="1"/>
     </row>
-    <row r="142" spans="2:2">
+    <row r="142" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B142" s="1"/>
     </row>
-    <row r="143" spans="2:2">
+    <row r="143" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B143" s="1"/>
     </row>
-    <row r="144" spans="2:2">
+    <row r="144" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B144" s="1"/>
     </row>
-    <row r="145" spans="2:2">
+    <row r="145" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B145" s="1"/>
     </row>
-    <row r="146" spans="2:2">
+    <row r="146" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B146" s="1"/>
     </row>
-    <row r="147" spans="2:2">
+    <row r="147" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B147" s="1"/>
     </row>
-    <row r="148" spans="2:2">
+    <row r="148" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B148" s="1"/>
     </row>
-    <row r="149" spans="2:2">
+    <row r="149" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B149" s="1"/>
     </row>
-    <row r="150" spans="2:2">
+    <row r="150" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B150" s="1"/>
     </row>
-    <row r="151" spans="2:2">
+    <row r="151" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B151" s="1"/>
     </row>
-    <row r="152" spans="2:2">
+    <row r="152" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B152" s="1"/>
     </row>
-    <row r="153" spans="2:2">
+    <row r="153" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B153" s="1"/>
     </row>
-    <row r="154" spans="2:2">
+    <row r="154" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B154" s="1"/>
     </row>
-    <row r="155" spans="2:2">
+    <row r="155" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B155" s="1"/>
     </row>
-    <row r="156" spans="2:2">
+    <row r="156" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B156" s="1"/>
     </row>
-    <row r="157" spans="2:2">
+    <row r="157" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B157" s="1"/>
     </row>
-    <row r="158" spans="2:2">
+    <row r="158" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B158" s="1"/>
     </row>
-    <row r="159" spans="2:2">
+    <row r="159" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B159" s="1"/>
     </row>
-    <row r="160" spans="2:2">
+    <row r="160" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B160" s="1"/>
     </row>
-    <row r="161" spans="2:2">
+    <row r="161" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B161" s="1"/>
     </row>
-    <row r="162" spans="2:2">
+    <row r="162" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B162" s="1"/>
     </row>
-    <row r="163" spans="2:2">
+    <row r="163" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B163" s="1"/>
     </row>
-    <row r="164" spans="2:2">
+    <row r="164" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B164" s="1"/>
     </row>
-    <row r="165" spans="2:2">
+    <row r="165" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B165" s="1"/>
     </row>
-    <row r="166" spans="2:2">
+    <row r="166" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B166" s="1"/>
     </row>
-    <row r="167" spans="2:2">
+    <row r="167" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B167" s="1"/>
     </row>
-    <row r="168" spans="2:2">
+    <row r="168" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B168" s="1"/>
     </row>
-    <row r="169" spans="2:2">
+    <row r="169" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B169" s="1"/>
     </row>
-    <row r="170" spans="2:2">
+    <row r="170" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B170" s="1"/>
     </row>
-    <row r="171" spans="2:2">
+    <row r="171" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B171" s="1"/>
     </row>
-    <row r="172" spans="2:2">
+    <row r="172" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B172" s="1"/>
     </row>
-    <row r="173" spans="2:2">
+    <row r="173" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B173" s="1"/>
     </row>
-    <row r="174" spans="2:2">
+    <row r="174" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B174" s="1"/>
     </row>
-    <row r="175" spans="2:2">
+    <row r="175" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B175" s="1"/>
     </row>
-    <row r="176" spans="2:2">
+    <row r="176" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B176" s="1"/>
     </row>
-    <row r="177" spans="2:2">
+    <row r="177" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B177" s="1"/>
     </row>
-    <row r="178" spans="2:2">
+    <row r="178" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B178" s="1"/>
     </row>
-    <row r="179" spans="2:2">
+    <row r="179" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B179" s="1"/>
     </row>
-    <row r="180" spans="2:2">
+    <row r="180" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B180" s="1"/>
     </row>
-    <row r="181" spans="2:2">
+    <row r="181" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B181" s="1"/>
     </row>
-    <row r="182" spans="2:2">
+    <row r="182" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B182" s="1"/>
     </row>
-    <row r="183" spans="2:2">
+    <row r="183" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B183" s="1"/>
     </row>
-    <row r="184" spans="2:2">
+    <row r="184" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B184" s="1"/>
     </row>
-    <row r="185" spans="2:2">
+    <row r="185" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B185" s="1"/>
     </row>
-    <row r="186" spans="2:2">
+    <row r="186" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B186" s="1"/>
     </row>
-    <row r="187" spans="2:2">
+    <row r="187" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B187" s="1"/>
     </row>
-    <row r="188" spans="2:2">
+    <row r="188" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B188" s="1"/>
     </row>
-    <row r="189" spans="2:2">
+    <row r="189" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B189" s="1"/>
     </row>
-    <row r="190" spans="2:2">
+    <row r="190" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B190" s="1"/>
     </row>
-    <row r="191" spans="2:2">
+    <row r="191" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B191" s="1"/>
     </row>
-    <row r="192" spans="2:2">
+    <row r="192" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B192" s="1"/>
     </row>
-    <row r="193" spans="2:2">
+    <row r="193" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B193" s="1"/>
     </row>
-    <row r="194" spans="2:2">
+    <row r="194" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="2:2">
+    <row r="195" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="2:2">
+    <row r="196" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="2:2">
+    <row r="197" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="2:2">
+    <row r="198" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="2:2">
+    <row r="199" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="2:2">
+    <row r="200" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="2:2">
+    <row r="201" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B201" s="1"/>
     </row>
-    <row r="202" spans="2:2">
+    <row r="202" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="2:2">
+    <row r="203" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="2:2">
+    <row r="204" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B204" s="1"/>
     </row>
-    <row r="205" spans="2:2">
+    <row r="205" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B205" s="1"/>
     </row>
-    <row r="206" spans="2:2">
+    <row r="206" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="2:2">
+    <row r="207" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="2:2">
+    <row r="208" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="2:2">
+    <row r="209" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B209" s="1"/>
     </row>
-    <row r="210" spans="2:2">
+    <row r="210" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="2:2">
+    <row r="211" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="2:2">
+    <row r="212" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="2:2">
+    <row r="213" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="2:2">
+    <row r="214" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="2:2">
+    <row r="215" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="2:2">
+    <row r="216" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="2:2">
+    <row r="217" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="2:2">
+    <row r="218" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B218" s="1"/>
     </row>
-    <row r="219" spans="2:2">
+    <row r="219" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B219" s="1"/>
     </row>
-    <row r="220" spans="2:2">
+    <row r="220" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B220" s="1"/>
     </row>
-    <row r="221" spans="2:2">
+    <row r="221" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B221" s="1"/>
     </row>
-    <row r="222" spans="2:2">
+    <row r="222" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B222" s="1"/>
     </row>
-    <row r="223" spans="2:2">
+    <row r="223" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B223" s="1"/>
     </row>
-    <row r="224" spans="2:2">
+    <row r="224" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B224" s="1"/>
     </row>
-    <row r="225" spans="2:2">
+    <row r="225" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B225" s="1"/>
     </row>
-    <row r="226" spans="2:2">
+    <row r="226" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B226" s="1"/>
     </row>
-    <row r="227" spans="2:2">
+    <row r="227" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B227" s="1"/>
     </row>
-    <row r="228" spans="2:2">
+    <row r="228" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B228" s="1"/>
     </row>
-    <row r="229" spans="2:2">
+    <row r="229" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B229" s="1"/>
     </row>
-    <row r="230" spans="2:2">
+    <row r="230" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B230" s="1"/>
     </row>
-    <row r="231" spans="2:2">
+    <row r="231" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B231" s="1"/>
     </row>
-    <row r="232" spans="2:2">
+    <row r="232" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B232" s="1"/>
     </row>
-    <row r="233" spans="2:2">
+    <row r="233" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B233" s="1"/>
     </row>
-    <row r="234" spans="2:2">
+    <row r="234" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B234" s="1"/>
     </row>
-    <row r="235" spans="2:2">
+    <row r="235" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B235" s="1"/>
     </row>
-    <row r="236" spans="2:2">
+    <row r="236" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B236" s="1"/>
     </row>
-    <row r="237" spans="2:2">
+    <row r="237" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B237" s="1"/>
     </row>
-    <row r="238" spans="2:2">
+    <row r="238" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B238" s="1"/>
     </row>
-    <row r="239" spans="2:2">
+    <row r="239" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B239" s="1"/>
     </row>
-    <row r="240" spans="2:2">
+    <row r="240" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B240" s="1"/>
     </row>
-    <row r="241" spans="2:2">
+    <row r="241" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B241" s="1"/>
     </row>
-    <row r="242" spans="2:2">
+    <row r="242" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B242" s="1"/>
     </row>
-    <row r="243" spans="2:2">
+    <row r="243" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B243" s="1"/>
     </row>
-    <row r="244" spans="2:2">
+    <row r="244" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B244" s="1"/>
     </row>
-    <row r="245" spans="2:2">
+    <row r="245" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B245" s="1"/>
     </row>
-    <row r="246" spans="2:2">
+    <row r="246" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B246" s="1"/>
     </row>
-    <row r="247" spans="2:2">
+    <row r="247" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B247" s="1"/>
     </row>
-    <row r="248" spans="2:2">
+    <row r="248" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B248" s="1"/>
     </row>
-    <row r="249" spans="2:2">
+    <row r="249" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B249" s="1"/>
     </row>
-    <row r="250" spans="2:2">
+    <row r="250" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B250" s="1"/>
     </row>
-    <row r="251" spans="2:2">
+    <row r="251" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B251" s="1"/>
     </row>
-    <row r="252" spans="2:2">
+    <row r="252" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B252" s="1"/>
     </row>
-    <row r="253" spans="2:2">
+    <row r="253" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B253" s="1"/>
     </row>
-    <row r="254" spans="2:2">
+    <row r="254" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B254" s="1"/>
     </row>
-    <row r="255" spans="2:2">
+    <row r="255" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B255" s="1"/>
     </row>
-    <row r="256" spans="2:2">
+    <row r="256" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B256" s="1"/>
     </row>
-    <row r="257" spans="2:2">
+    <row r="257" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B257" s="1"/>
     </row>
-    <row r="258" spans="2:2">
+    <row r="258" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B258" s="1"/>
     </row>
-    <row r="259" spans="2:2">
+    <row r="259" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B259" s="1"/>
     </row>
-    <row r="260" spans="2:2">
+    <row r="260" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B260" s="1"/>
     </row>
-    <row r="261" spans="2:2">
+    <row r="261" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B261" s="1"/>
     </row>
-    <row r="262" spans="2:2">
+    <row r="262" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B262" s="1"/>
     </row>
-    <row r="263" spans="2:2">
+    <row r="263" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B263" s="1"/>
     </row>
-    <row r="264" spans="2:2">
+    <row r="264" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B264" s="1"/>
     </row>
-    <row r="265" spans="2:2">
+    <row r="265" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B265" s="1"/>
     </row>
-    <row r="266" spans="2:2">
+    <row r="266" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B266" s="1"/>
     </row>
-    <row r="267" spans="2:2">
+    <row r="267" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B267" s="1"/>
     </row>
-    <row r="268" spans="2:2">
+    <row r="268" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B268" s="1"/>
     </row>
-    <row r="269" spans="2:2">
+    <row r="269" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B269" s="1"/>
     </row>
-    <row r="270" spans="2:2">
+    <row r="270" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B270" s="1"/>
     </row>
-    <row r="271" spans="2:2">
+    <row r="271" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B271" s="1"/>
     </row>
-    <row r="272" spans="2:2">
+    <row r="272" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B272" s="1"/>
     </row>
-    <row r="273" spans="2:2">
+    <row r="273" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B273" s="1"/>
     </row>
-    <row r="274" spans="2:2">
+    <row r="274" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B274" s="1"/>
     </row>
-    <row r="275" spans="2:2">
+    <row r="275" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B275" s="1"/>
     </row>
-    <row r="276" spans="2:2">
+    <row r="276" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B276" s="1"/>
     </row>
-    <row r="277" spans="2:2">
+    <row r="277" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B277" s="1"/>
     </row>
-    <row r="278" spans="2:2">
+    <row r="278" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B278" s="1"/>
     </row>
-    <row r="279" spans="2:2">
+    <row r="279" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B279" s="1"/>
     </row>
-    <row r="280" spans="2:2">
+    <row r="280" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B280" s="1"/>
     </row>
-    <row r="281" spans="2:2">
+    <row r="281" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B281" s="1"/>
     </row>
-    <row r="282" spans="2:2">
+    <row r="282" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B282" s="1"/>
     </row>
-    <row r="283" spans="2:2">
+    <row r="283" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B283" s="1"/>
     </row>
-    <row r="284" spans="2:2">
+    <row r="284" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B284" s="1"/>
     </row>
-    <row r="285" spans="2:2">
+    <row r="285" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B285" s="1"/>
     </row>
-    <row r="286" spans="2:2">
+    <row r="286" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B286" s="1"/>
     </row>
-    <row r="287" spans="2:2">
+    <row r="287" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B287" s="1"/>
     </row>
-    <row r="288" spans="2:2">
+    <row r="288" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B288" s="1"/>
     </row>
-    <row r="289" spans="2:2">
+    <row r="289" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B289" s="1"/>
     </row>
-    <row r="290" spans="2:2">
+    <row r="290" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B290" s="1"/>
     </row>
-    <row r="291" spans="2:2">
+    <row r="291" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B291" s="1"/>
     </row>
-    <row r="292" spans="2:2">
+    <row r="292" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B292" s="1"/>
     </row>
-    <row r="293" spans="2:2">
+    <row r="293" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B293" s="1"/>
     </row>
-    <row r="294" spans="2:2">
+    <row r="294" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B294" s="1"/>
     </row>
-    <row r="295" spans="2:2">
+    <row r="295" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B295" s="1"/>
     </row>
-    <row r="296" spans="2:2">
+    <row r="296" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B296" s="1"/>
     </row>
-    <row r="297" spans="2:2">
+    <row r="297" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B297" s="1"/>
     </row>
-    <row r="298" spans="2:2">
+    <row r="298" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B298" s="1"/>
     </row>
-    <row r="299" spans="2:2">
+    <row r="299" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B299" s="1"/>
     </row>
-    <row r="300" spans="2:2">
+    <row r="300" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B300" s="1"/>
     </row>
-    <row r="301" spans="2:2">
+    <row r="301" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B301" s="1"/>
     </row>
-    <row r="302" spans="2:2">
+    <row r="302" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B302" s="1"/>
     </row>
-    <row r="303" spans="2:2">
+    <row r="303" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B303" s="1"/>
     </row>
-    <row r="304" spans="2:2">
+    <row r="304" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B304" s="1"/>
     </row>
-    <row r="305" spans="2:2">
+    <row r="305" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B305" s="1"/>
     </row>
-    <row r="306" spans="2:2">
+    <row r="306" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B306" s="1"/>
     </row>
-    <row r="307" spans="2:2">
+    <row r="307" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B307" s="1"/>
     </row>
-    <row r="308" spans="2:2">
+    <row r="308" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B308" s="1"/>
     </row>
-    <row r="309" spans="2:2">
+    <row r="309" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B309" s="1"/>
     </row>
-    <row r="310" spans="2:2">
+    <row r="310" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B310" s="1"/>
     </row>
-    <row r="311" spans="2:2">
+    <row r="311" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B311" s="1"/>
     </row>
-    <row r="312" spans="2:2">
+    <row r="312" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B312" s="1"/>
     </row>
-    <row r="313" spans="2:2">
+    <row r="313" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B313" s="1"/>
     </row>
-    <row r="314" spans="2:2">
+    <row r="314" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B314" s="1"/>
     </row>
-    <row r="315" spans="2:2">
+    <row r="315" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B315" s="1"/>
     </row>
-    <row r="316" spans="2:2">
+    <row r="316" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B316" s="1"/>
     </row>
-    <row r="317" spans="2:2">
+    <row r="317" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B317" s="1"/>
     </row>
-    <row r="318" spans="2:2">
+    <row r="318" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B318" s="1"/>
     </row>
-    <row r="319" spans="2:2">
+    <row r="319" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B319" s="1"/>
     </row>
-    <row r="320" spans="2:2">
+    <row r="320" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B320" s="1"/>
     </row>
-    <row r="321" spans="2:2">
+    <row r="321" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B321" s="1"/>
     </row>
-    <row r="322" spans="2:2">
+    <row r="322" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B322" s="1"/>
     </row>
-    <row r="323" spans="2:2">
+    <row r="323" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B323" s="1"/>
     </row>
-    <row r="324" spans="2:2">
+    <row r="324" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B324" s="1"/>
     </row>
-    <row r="325" spans="2:2">
+    <row r="325" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B325" s="1"/>
     </row>
-    <row r="326" spans="2:2">
+    <row r="326" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B326" s="1"/>
     </row>
-    <row r="327" spans="2:2">
+    <row r="327" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B327" s="1"/>
     </row>
-    <row r="328" spans="2:2">
+    <row r="328" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B328" s="1"/>
     </row>
-    <row r="329" spans="2:2">
+    <row r="329" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B329" s="1"/>
     </row>
-    <row r="330" spans="2:2">
+    <row r="330" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B330" s="1"/>
     </row>
-    <row r="331" spans="2:2">
+    <row r="331" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B331" s="1"/>
     </row>
   </sheetData>

</xml_diff>